<commit_message>
Export: fill Excel templates via {{placeholders}} with dynamic truck blocks
Adds placeholder replacement so the exact Excel layout/borders remain unchanged and supports variable truck sections even when truck fields span multiple rows.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Formats/Export/Commercial Invoice.xlsx
+++ b/Formats/Export/Commercial Invoice.xlsx
@@ -1,21 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4507"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\NIKHI\Desktop\Order Processing JLD\Formats\Export\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="120" yWindow="120" windowWidth="21495" windowHeight="9975" activeTab="1"/>
+    <workbookView xWindow="120" yWindow="120" windowWidth="21492" windowHeight="9972" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Tax Invoice" sheetId="3" r:id="rId1"/>
     <sheet name="Packing List" sheetId="5" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="125725"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="115">
   <si>
     <t>IEC</t>
   </si>
@@ -149,24 +154,9 @@
     <t>ICICINBBCTS</t>
   </si>
   <si>
-    <t>ARIHANT INFRASTRUCTURE LIMITED</t>
-  </si>
-  <si>
     <t>NEPAL</t>
   </si>
   <si>
-    <t>MAIN ROAD, BIRATNAGAR, NEPAL</t>
-  </si>
-  <si>
-    <t>PAN NO: 303714123</t>
-  </si>
-  <si>
-    <t>EXIM CODE : 3037141230158NP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TO THE ORDER OF HIMALAYAN BANK LTD </t>
-  </si>
-  <si>
     <t>DOCUMENTRY CREDIT NUMBER : HBLIRIC05801794</t>
   </si>
   <si>
@@ -180,9 +170,6 @@
   </si>
   <si>
     <t>SUNSARI, NEPAL VIA BIRATNAGAR CUSTOMS OFFICE, NEPAL</t>
-  </si>
-  <si>
-    <t>PO NO. HO/PO.19/80-81 Date : 01-03-2024</t>
   </si>
   <si>
     <t>BIKANER (RAJASTHAN), INDIA</t>
@@ -305,21 +292,12 @@
     <t>INDUSTRIAL RAW MATERIAL FOR TILES INDUSTRY</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Payment Terms : 180 DAYS AT SIGHT                                                                                                      2. Delivery Terms : CPT JOGBANI LAND PORT, INDIA                                                      3. Delivery Frrom : Tehsil Shrimodhopur, Dist. Neem Ka Thana, Raj.-332701                                                  </t>
-  </si>
-  <si>
     <t xml:space="preserve">     Packed In Small Bags </t>
   </si>
   <si>
     <t>Original Copy</t>
   </si>
   <si>
-    <t>NEPAL/EXP-045</t>
-  </si>
-  <si>
-    <t>24/05/2024</t>
-  </si>
-  <si>
     <t>Truck No. : PB10JF9339, PB10HZ9639</t>
   </si>
   <si>
@@ -330,6 +308,39 @@
   </si>
   <si>
     <t>20811 Dt: 23/05/2024,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     Total No. Of Bags = 1680 Bags</t>
+  </si>
+  <si>
+    <t>23-05-2024</t>
+  </si>
+  <si>
+    <t>(840 Bags)</t>
+  </si>
+  <si>
+    <t>PB10HZ9639</t>
+  </si>
+  <si>
+    <t>Our PI NO. 107 Date: 04-06-2024</t>
+  </si>
+  <si>
+    <t>Shipping Bill No. &amp; Dt : 1221042 Dt: 28-MAY-2024</t>
+  </si>
+  <si>
+    <t>{{INVOICE_NO}}</t>
+  </si>
+  <si>
+    <t>{{INVOICE_DATE}}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Payment Terms : 180 DAYS AT SIGHT                                                                                                      2. Delivery Terms : CPT JOGBANI LAND PORT, INDIA                                                      3. Delivery From : Tehsil Shrimodhopur, Dist. Neem Ka Thana, Raj.-332701                                                  </t>
+  </si>
+  <si>
+    <t>{{CONSIGNEE}}</t>
+  </si>
+  <si>
+    <t>{{CONSIGNEE_ADDRESS}}</t>
   </si>
   <si>
     <r>
@@ -344,39 +355,51 @@
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
-      <t>FOUR LAKH THIRTY SEVEN THOUSAND EIGHT HUNDRED NINTY TWO ONLY</t>
+      <t>{{AMOUNT_IN_WORDS}}</t>
     </r>
   </si>
   <si>
-    <t xml:space="preserve">     Total No. Of Bags = 1680 Bags</t>
-  </si>
-  <si>
-    <t>PB10JF9339</t>
-  </si>
-  <si>
-    <t>23-05-2024</t>
-  </si>
-  <si>
-    <t>(840 Bags)</t>
-  </si>
-  <si>
-    <t>PB10HZ9639</t>
-  </si>
-  <si>
-    <t>Our PI NO. 107 Date: 04-06-2024</t>
-  </si>
-  <si>
-    <t>Shipping Bill No. &amp; Dt : 1221042 Dt: 28-MAY-2024</t>
+    <t>{{NOTIFY_APPLICANT}}</t>
+  </si>
+  <si>
+    <t>{{NOTIFY_APPLICANT_ADDRESS}}</t>
+  </si>
+  <si>
+    <t>PAN NO: {{PAN_NO}}</t>
+  </si>
+  <si>
+    <t>EXIM CODE : {{EXIM_CODE}}</t>
+  </si>
+  <si>
+    <t>{{BUYER_ORDER_NO}} Date : {{BUYER_ORDER_DATE}}</t>
+  </si>
+  <si>
+    <t>{{RATE_PER_MT}}</t>
+  </si>
+  <si>
+    <t>DOCUMENTRY CREDIT NUMBER : {{DOCUMENTRY_CREDIT_NO}}</t>
+  </si>
+  <si>
+    <t>{{TRUCK_NO}}</t>
+  </si>
+  <si>
+    <t>{{LR_NO}}</t>
+  </si>
+  <si>
+    <t>{{QTY_IN_MT}}</t>
+  </si>
+  <si>
+    <t>{{DATE}}</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="37">
+  <fonts count="37" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1357,251 +1380,78 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="41" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="35" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="36" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="37" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="17" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="18" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="15" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="20" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="29" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="32" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="34" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="8" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="21" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="33" fillId="0" borderId="21" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="33" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="33" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
@@ -1667,92 +1517,380 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="8" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="21" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="35" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="36" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="37" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="17" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="18" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="15" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="20" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="29" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="32" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="23" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="35" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="36" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="37" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="21" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="6" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="19" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="11" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="34" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="2" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="4" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="23" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="11" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="13" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="39" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="40" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="31" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="29" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="32" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="19" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="38" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="20" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="7" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="20" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="7" xfId="37" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="37" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="20" xfId="37" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="35" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="36" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="37" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="17" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1783,121 +1921,6 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="31" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="29" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="32" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="19" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="38" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="20" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="7" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="20" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="7" xfId="37" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="37" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="20" xfId="37" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="11" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="13" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="39" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="40" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="23" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="21" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="6" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="19" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="11" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="2" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="4" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="23" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="38">
     <cellStyle name="Followed Hyperlink" xfId="4" builtinId="9" hidden="1"/>
@@ -1941,6 +1964,14 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -1987,7 +2018,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -2019,9 +2050,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -2053,6 +2085,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -2228,342 +2261,342 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G48"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.375" customWidth="1"/>
-    <col min="3" max="3" width="17.125" customWidth="1"/>
+    <col min="1" max="1" width="19.59765625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.3984375" customWidth="1"/>
+    <col min="3" max="3" width="17.09765625" customWidth="1"/>
     <col min="4" max="4" width="11" customWidth="1"/>
     <col min="5" max="5" width="9.5" customWidth="1"/>
-    <col min="6" max="6" width="10.875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.75" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.8984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.69921875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="35.25" thickBot="1">
-      <c r="A1" s="82" t="s">
+    <row r="1" spans="1:7" ht="35.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="213" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="82"/>
-      <c r="C1" s="82"/>
-      <c r="D1" s="82"/>
-      <c r="E1" s="82"/>
-      <c r="F1" s="82"/>
-      <c r="G1" s="82"/>
-    </row>
-    <row r="2" spans="1:7" ht="18.75" thickBot="1">
+      <c r="B1" s="213"/>
+      <c r="C1" s="213"/>
+      <c r="D1" s="213"/>
+      <c r="E1" s="213"/>
+      <c r="F1" s="213"/>
+      <c r="G1" s="213"/>
+    </row>
+    <row r="2" spans="1:7" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="10" t="s">
         <v>14</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
-      <c r="E2" s="83" t="s">
-        <v>94</v>
-      </c>
-      <c r="F2" s="84"/>
-      <c r="G2" s="85"/>
-    </row>
-    <row r="3" spans="1:7" ht="15" thickBot="1">
-      <c r="A3" s="95" t="s">
-        <v>73</v>
-      </c>
-      <c r="B3" s="95"/>
-      <c r="C3" s="95"/>
-      <c r="D3" s="95"/>
-      <c r="E3" s="95"/>
-      <c r="F3" s="95"/>
-      <c r="G3" s="96"/>
-    </row>
-    <row r="4" spans="1:7" ht="15.75">
+      <c r="E2" s="214" t="s">
+        <v>87</v>
+      </c>
+      <c r="F2" s="215"/>
+      <c r="G2" s="216"/>
+    </row>
+    <row r="3" spans="1:7" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="226" t="s">
+        <v>67</v>
+      </c>
+      <c r="B3" s="226"/>
+      <c r="C3" s="226"/>
+      <c r="D3" s="226"/>
+      <c r="E3" s="226"/>
+      <c r="F3" s="226"/>
+      <c r="G3" s="227"/>
+    </row>
+    <row r="4" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B4" s="77" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="86" t="s">
+      <c r="C4" s="217" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="87"/>
-      <c r="E4" s="86" t="s">
+      <c r="D4" s="218"/>
+      <c r="E4" s="217" t="s">
         <v>3</v>
       </c>
-      <c r="F4" s="88"/>
-      <c r="G4" s="89"/>
-    </row>
-    <row r="5" spans="1:7" ht="16.5">
+      <c r="F4" s="219"/>
+      <c r="G4" s="220"/>
+    </row>
+    <row r="5" spans="1:7" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>4</v>
       </c>
       <c r="B5" s="79" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="90" t="s">
-        <v>95</v>
-      </c>
-      <c r="D5" s="91"/>
-      <c r="E5" s="92" t="s">
+      <c r="C5" s="221" t="s">
+        <v>98</v>
+      </c>
+      <c r="D5" s="222"/>
+      <c r="E5" s="223" t="s">
+        <v>99</v>
+      </c>
+      <c r="F5" s="224"/>
+      <c r="G5" s="225"/>
+    </row>
+    <row r="6" spans="1:7" ht="15" x14ac:dyDescent="0.25">
+      <c r="A6" s="182" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="185"/>
+      <c r="C6" s="205" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6" s="206"/>
+      <c r="E6" s="206"/>
+      <c r="F6" s="206"/>
+      <c r="G6" s="207"/>
+    </row>
+    <row r="7" spans="1:7" ht="15" x14ac:dyDescent="0.25">
+      <c r="A7" s="208" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="209"/>
+      <c r="C7" s="210" t="s">
+        <v>108</v>
+      </c>
+      <c r="D7" s="211"/>
+      <c r="E7" s="211"/>
+      <c r="F7" s="211"/>
+      <c r="G7" s="212"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="195" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="110"/>
+      <c r="C8" s="202"/>
+      <c r="D8" s="203"/>
+      <c r="E8" s="203"/>
+      <c r="F8" s="203"/>
+      <c r="G8" s="204"/>
+    </row>
+    <row r="9" spans="1:7" ht="15" x14ac:dyDescent="0.25">
+      <c r="A9" s="195" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="111"/>
+      <c r="C9" s="196" t="s">
+        <v>22</v>
+      </c>
+      <c r="D9" s="197"/>
+      <c r="E9" s="197"/>
+      <c r="F9" s="197"/>
+      <c r="G9" s="198"/>
+    </row>
+    <row r="10" spans="1:7" ht="15" x14ac:dyDescent="0.25">
+      <c r="A10" s="195" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" s="111"/>
+      <c r="C10" s="199" t="s">
         <v>96</v>
       </c>
-      <c r="F5" s="93"/>
-      <c r="G5" s="94"/>
-    </row>
-    <row r="6" spans="1:7" ht="15.75">
-      <c r="A6" s="97" t="s">
-        <v>16</v>
-      </c>
-      <c r="B6" s="98"/>
-      <c r="C6" s="99" t="s">
-        <v>19</v>
-      </c>
-      <c r="D6" s="100"/>
-      <c r="E6" s="100"/>
-      <c r="F6" s="100"/>
-      <c r="G6" s="101"/>
-    </row>
-    <row r="7" spans="1:7" ht="15.75">
-      <c r="A7" s="102" t="s">
-        <v>17</v>
-      </c>
-      <c r="B7" s="103"/>
-      <c r="C7" s="104" t="s">
-        <v>55</v>
-      </c>
-      <c r="D7" s="105"/>
-      <c r="E7" s="105"/>
-      <c r="F7" s="105"/>
-      <c r="G7" s="106"/>
-    </row>
-    <row r="8" spans="1:7">
-      <c r="A8" s="107" t="s">
-        <v>18</v>
-      </c>
-      <c r="B8" s="108"/>
-      <c r="C8" s="109"/>
-      <c r="D8" s="110"/>
-      <c r="E8" s="110"/>
-      <c r="F8" s="110"/>
-      <c r="G8" s="111"/>
-    </row>
-    <row r="9" spans="1:7" ht="15.75">
-      <c r="A9" s="107" t="s">
-        <v>20</v>
-      </c>
-      <c r="B9" s="112"/>
-      <c r="C9" s="113" t="s">
-        <v>22</v>
-      </c>
-      <c r="D9" s="114"/>
-      <c r="E9" s="114"/>
-      <c r="F9" s="114"/>
-      <c r="G9" s="115"/>
-    </row>
-    <row r="10" spans="1:7" ht="15.75">
-      <c r="A10" s="107" t="s">
-        <v>21</v>
-      </c>
-      <c r="B10" s="112"/>
-      <c r="C10" s="116" t="s">
+      <c r="D10" s="200"/>
+      <c r="E10" s="200"/>
+      <c r="F10" s="200"/>
+      <c r="G10" s="201"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="195" t="s">
+        <v>23</v>
+      </c>
+      <c r="B11" s="111"/>
+      <c r="C11" s="202"/>
+      <c r="D11" s="203"/>
+      <c r="E11" s="203"/>
+      <c r="F11" s="203"/>
+      <c r="G11" s="204"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="182" t="s">
+        <v>24</v>
+      </c>
+      <c r="B12" s="183"/>
+      <c r="C12" s="184" t="s">
+        <v>25</v>
+      </c>
+      <c r="D12" s="185"/>
+      <c r="E12" s="185"/>
+      <c r="F12" s="185"/>
+      <c r="G12" s="186"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="187" t="s">
+        <v>101</v>
+      </c>
+      <c r="B13" s="188"/>
+      <c r="C13" s="189" t="s">
+        <v>104</v>
+      </c>
+      <c r="D13" s="190"/>
+      <c r="E13" s="190"/>
+      <c r="F13" s="190"/>
+      <c r="G13" s="191"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="180" t="s">
+        <v>102</v>
+      </c>
+      <c r="B14" s="181"/>
+      <c r="C14" s="192" t="s">
+        <v>105</v>
+      </c>
+      <c r="D14" s="193"/>
+      <c r="E14" s="193"/>
+      <c r="F14" s="193"/>
+      <c r="G14" s="194"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="175" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" s="176"/>
+      <c r="C15" s="177" t="s">
+        <v>106</v>
+      </c>
+      <c r="D15" s="178"/>
+      <c r="E15" s="178"/>
+      <c r="F15" s="178"/>
+      <c r="G15" s="179"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="180"/>
+      <c r="B16" s="181"/>
+      <c r="C16" s="177" t="s">
         <v>107</v>
       </c>
-      <c r="D10" s="117"/>
-      <c r="E10" s="117"/>
-      <c r="F10" s="117"/>
-      <c r="G10" s="118"/>
-    </row>
-    <row r="11" spans="1:7">
-      <c r="A11" s="107" t="s">
-        <v>23</v>
-      </c>
-      <c r="B11" s="112"/>
-      <c r="C11" s="109"/>
-      <c r="D11" s="110"/>
-      <c r="E11" s="110"/>
-      <c r="F11" s="110"/>
-      <c r="G11" s="111"/>
-    </row>
-    <row r="12" spans="1:7">
-      <c r="A12" s="97" t="s">
-        <v>24</v>
-      </c>
-      <c r="B12" s="119"/>
-      <c r="C12" s="120" t="s">
-        <v>25</v>
-      </c>
-      <c r="D12" s="98"/>
-      <c r="E12" s="98"/>
-      <c r="F12" s="98"/>
-      <c r="G12" s="121"/>
-    </row>
-    <row r="13" spans="1:7">
-      <c r="A13" s="122" t="s">
-        <v>49</v>
-      </c>
-      <c r="B13" s="123"/>
-      <c r="C13" s="124" t="s">
-        <v>44</v>
-      </c>
-      <c r="D13" s="125"/>
-      <c r="E13" s="125"/>
-      <c r="F13" s="125"/>
-      <c r="G13" s="126"/>
-    </row>
-    <row r="14" spans="1:7">
-      <c r="A14" s="127" t="s">
-        <v>45</v>
-      </c>
-      <c r="B14" s="128"/>
-      <c r="C14" s="129" t="s">
-        <v>46</v>
-      </c>
-      <c r="D14" s="130"/>
-      <c r="E14" s="130"/>
-      <c r="F14" s="130"/>
-      <c r="G14" s="131"/>
-    </row>
-    <row r="15" spans="1:7">
-      <c r="A15" s="138" t="s">
-        <v>14</v>
-      </c>
-      <c r="B15" s="139"/>
-      <c r="C15" s="140" t="s">
-        <v>47</v>
-      </c>
-      <c r="D15" s="141"/>
-      <c r="E15" s="141"/>
-      <c r="F15" s="141"/>
-      <c r="G15" s="142"/>
-    </row>
-    <row r="16" spans="1:7">
-      <c r="A16" s="127"/>
-      <c r="B16" s="128"/>
-      <c r="C16" s="140" t="s">
-        <v>48</v>
-      </c>
-      <c r="D16" s="141"/>
-      <c r="E16" s="141"/>
-      <c r="F16" s="141"/>
-      <c r="G16" s="142"/>
-    </row>
-    <row r="17" spans="1:7">
+      <c r="D16" s="178"/>
+      <c r="E16" s="178"/>
+      <c r="F16" s="178"/>
+      <c r="G16" s="179"/>
+    </row>
+    <row r="17" spans="1:7" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A17" s="40" t="s">
         <v>26</v>
       </c>
       <c r="B17" s="49" t="s">
         <v>27</v>
       </c>
-      <c r="C17" s="132" t="s">
+      <c r="C17" s="169" t="s">
         <v>31</v>
       </c>
-      <c r="D17" s="133"/>
-      <c r="E17" s="133"/>
-      <c r="F17" s="133"/>
-      <c r="G17" s="134"/>
-    </row>
-    <row r="18" spans="1:7" ht="44.25" customHeight="1">
+      <c r="D17" s="170"/>
+      <c r="E17" s="170"/>
+      <c r="F17" s="170"/>
+      <c r="G17" s="171"/>
+    </row>
+    <row r="18" spans="1:7" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="41" t="s">
         <v>30</v>
       </c>
       <c r="B18" s="50" t="s">
-        <v>56</v>
-      </c>
-      <c r="C18" s="135" t="s">
-        <v>92</v>
-      </c>
-      <c r="D18" s="136"/>
-      <c r="E18" s="136"/>
-      <c r="F18" s="136"/>
-      <c r="G18" s="137"/>
-    </row>
-    <row r="19" spans="1:7">
+        <v>50</v>
+      </c>
+      <c r="C18" s="172" t="s">
+        <v>100</v>
+      </c>
+      <c r="D18" s="173"/>
+      <c r="E18" s="173"/>
+      <c r="F18" s="173"/>
+      <c r="G18" s="174"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="42" t="s">
         <v>28</v>
       </c>
       <c r="B19" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="C19" s="143" t="s">
-        <v>97</v>
-      </c>
-      <c r="D19" s="144"/>
-      <c r="E19" s="144"/>
-      <c r="F19" s="144"/>
-      <c r="G19" s="145"/>
-    </row>
-    <row r="20" spans="1:7">
+      <c r="C19" s="139" t="s">
+        <v>88</v>
+      </c>
+      <c r="D19" s="140"/>
+      <c r="E19" s="140"/>
+      <c r="F19" s="140"/>
+      <c r="G19" s="141"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="41" t="s">
         <v>6</v>
       </c>
       <c r="B20" s="78" t="s">
-        <v>45</v>
-      </c>
-      <c r="C20" s="146" t="s">
+        <v>44</v>
+      </c>
+      <c r="C20" s="142" t="s">
         <v>14</v>
       </c>
-      <c r="D20" s="147"/>
-      <c r="E20" s="147"/>
-      <c r="F20" s="147"/>
-      <c r="G20" s="148"/>
-    </row>
-    <row r="21" spans="1:7">
-      <c r="A21" s="218" t="s">
+      <c r="D20" s="143"/>
+      <c r="E20" s="143"/>
+      <c r="F20" s="143"/>
+      <c r="G20" s="144"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="88" t="s">
         <v>32</v>
       </c>
-      <c r="B21" s="219"/>
-      <c r="C21" s="212" t="s">
-        <v>99</v>
-      </c>
-      <c r="D21" s="213"/>
-      <c r="E21" s="213"/>
-      <c r="F21" s="213"/>
-      <c r="G21" s="214"/>
-    </row>
-    <row r="22" spans="1:7">
-      <c r="A22" s="220" t="s">
-        <v>54</v>
-      </c>
-      <c r="B22" s="221"/>
-      <c r="C22" s="215" t="s">
-        <v>100</v>
-      </c>
-      <c r="D22" s="216"/>
-      <c r="E22" s="216"/>
-      <c r="F22" s="216"/>
-      <c r="G22" s="217"/>
-    </row>
-    <row r="23" spans="1:7">
-      <c r="A23" s="220"/>
-      <c r="B23" s="221"/>
-      <c r="C23" s="146"/>
-      <c r="D23" s="147"/>
-      <c r="E23" s="147"/>
-      <c r="F23" s="147"/>
-      <c r="G23" s="148"/>
-    </row>
-    <row r="24" spans="1:7">
-      <c r="A24" s="169"/>
-      <c r="B24" s="170"/>
-      <c r="C24" s="225" t="s">
-        <v>108</v>
-      </c>
-      <c r="D24" s="226"/>
-      <c r="E24" s="226"/>
-      <c r="F24" s="226"/>
-      <c r="G24" s="227"/>
-    </row>
-    <row r="25" spans="1:7">
-      <c r="A25" s="203" t="s">
+      <c r="B21" s="89"/>
+      <c r="C21" s="82" t="s">
+        <v>90</v>
+      </c>
+      <c r="D21" s="83"/>
+      <c r="E21" s="83"/>
+      <c r="F21" s="83"/>
+      <c r="G21" s="84"/>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="90" t="s">
+        <v>49</v>
+      </c>
+      <c r="B22" s="91"/>
+      <c r="C22" s="85" t="s">
+        <v>91</v>
+      </c>
+      <c r="D22" s="86"/>
+      <c r="E22" s="86"/>
+      <c r="F22" s="86"/>
+      <c r="G22" s="87"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="90"/>
+      <c r="B23" s="91"/>
+      <c r="C23" s="142"/>
+      <c r="D23" s="143"/>
+      <c r="E23" s="143"/>
+      <c r="F23" s="143"/>
+      <c r="G23" s="144"/>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="165"/>
+      <c r="B24" s="166"/>
+      <c r="C24" s="96" t="s">
+        <v>97</v>
+      </c>
+      <c r="D24" s="97"/>
+      <c r="E24" s="97"/>
+      <c r="F24" s="97"/>
+      <c r="G24" s="98"/>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="92" t="s">
         <v>7</v>
       </c>
-      <c r="B25" s="223" t="s">
+      <c r="B25" s="94" t="s">
         <v>8</v>
       </c>
-      <c r="C25" s="149" t="s">
+      <c r="C25" s="145" t="s">
         <v>9</v>
       </c>
-      <c r="D25" s="150"/>
+      <c r="D25" s="146"/>
       <c r="E25" s="28" t="s">
         <v>10</v>
       </c>
@@ -2574,331 +2607,336 @@
         <v>12</v>
       </c>
     </row>
-    <row r="26" spans="1:7">
-      <c r="A26" s="222"/>
-      <c r="B26" s="224"/>
-      <c r="C26" s="151"/>
-      <c r="D26" s="152"/>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="93"/>
+      <c r="B26" s="95"/>
+      <c r="C26" s="147"/>
+      <c r="D26" s="148"/>
       <c r="E26" s="3" t="s">
         <v>13</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" ht="14.25" customHeight="1">
-      <c r="A27" s="203" t="s">
-        <v>51</v>
+        <v>48</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="92" t="s">
+        <v>46</v>
       </c>
       <c r="B27" s="31"/>
-      <c r="C27" s="156"/>
-      <c r="D27" s="157"/>
+      <c r="C27" s="152"/>
+      <c r="D27" s="153"/>
       <c r="E27" s="28"/>
       <c r="F27" s="28"/>
       <c r="G27" s="29"/>
     </row>
-    <row r="28" spans="1:7" ht="31.5" customHeight="1">
-      <c r="A28" s="204"/>
+    <row r="28" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="102"/>
       <c r="B28" s="80" t="s">
-        <v>98</v>
-      </c>
-      <c r="C28" s="154" t="s">
-        <v>91</v>
-      </c>
-      <c r="D28" s="155"/>
+        <v>89</v>
+      </c>
+      <c r="C28" s="150" t="s">
+        <v>85</v>
+      </c>
+      <c r="D28" s="151"/>
       <c r="E28" s="32"/>
       <c r="F28" s="33"/>
       <c r="G28" s="34"/>
     </row>
-    <row r="29" spans="1:7">
-      <c r="A29" s="204"/>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" s="102"/>
       <c r="B29" s="35"/>
-      <c r="C29" s="154" t="s">
-        <v>87</v>
-      </c>
-      <c r="D29" s="155"/>
+      <c r="C29" s="150" t="s">
+        <v>81</v>
+      </c>
+      <c r="D29" s="151"/>
       <c r="E29" s="32">
-        <f>42.28+41.93</f>
-        <v>84.210000000000008</v>
-      </c>
-      <c r="F29" s="33">
-        <v>5200</v>
-      </c>
-      <c r="G29" s="34">
+        <f>'Packing List'!G39</f>
+        <v>41.93</v>
+      </c>
+      <c r="F29" s="33" t="s">
+        <v>109</v>
+      </c>
+      <c r="G29" s="34" t="e">
         <f>E29*F29</f>
-        <v>437892.00000000006</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" ht="6.75" customHeight="1">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="7"/>
       <c r="B30" s="53" t="s">
         <v>14</v>
       </c>
-      <c r="C30" s="171"/>
-      <c r="D30" s="172"/>
+      <c r="C30" s="167"/>
+      <c r="D30" s="168"/>
       <c r="E30" s="36"/>
       <c r="F30" s="36"/>
       <c r="G30" s="8"/>
     </row>
-    <row r="31" spans="1:7">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="7"/>
-      <c r="B31" s="205" t="s">
-        <v>50</v>
-      </c>
-      <c r="C31" s="206"/>
-      <c r="D31" s="207"/>
+      <c r="B31" s="103" t="s">
+        <v>110</v>
+      </c>
+      <c r="C31" s="104"/>
+      <c r="D31" s="105"/>
       <c r="E31" s="51"/>
       <c r="F31" s="36"/>
       <c r="G31" s="8"/>
     </row>
-    <row r="32" spans="1:7">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="7"/>
-      <c r="B32" s="208" t="s">
-        <v>58</v>
-      </c>
-      <c r="C32" s="209"/>
-      <c r="D32" s="210"/>
+      <c r="B32" s="106" t="s">
+        <v>52</v>
+      </c>
+      <c r="C32" s="107"/>
+      <c r="D32" s="108"/>
       <c r="E32" s="51"/>
       <c r="F32" s="36"/>
       <c r="G32" s="8"/>
     </row>
-    <row r="33" spans="1:7">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="7"/>
-      <c r="B33" s="211" t="s">
-        <v>88</v>
-      </c>
-      <c r="C33" s="108"/>
-      <c r="D33" s="112"/>
+      <c r="B33" s="109" t="s">
+        <v>82</v>
+      </c>
+      <c r="C33" s="110"/>
+      <c r="D33" s="111"/>
       <c r="E33" s="51"/>
       <c r="F33" s="36"/>
       <c r="G33" s="8"/>
     </row>
-    <row r="34" spans="1:7">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="37"/>
-      <c r="B34" s="208" t="s">
-        <v>89</v>
-      </c>
-      <c r="C34" s="209"/>
-      <c r="D34" s="210"/>
+      <c r="B34" s="106" t="s">
+        <v>83</v>
+      </c>
+      <c r="C34" s="107"/>
+      <c r="D34" s="108"/>
       <c r="E34" s="51"/>
       <c r="F34" s="36"/>
       <c r="G34" s="8"/>
     </row>
-    <row r="35" spans="1:7" ht="30" customHeight="1">
+    <row r="35" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="37"/>
-      <c r="B35" s="200" t="s">
-        <v>59</v>
-      </c>
-      <c r="C35" s="201"/>
-      <c r="D35" s="202"/>
+      <c r="B35" s="99" t="s">
+        <v>53</v>
+      </c>
+      <c r="C35" s="100"/>
+      <c r="D35" s="101"/>
       <c r="E35" s="52"/>
       <c r="F35" s="38"/>
       <c r="G35" s="22"/>
     </row>
-    <row r="36" spans="1:7" ht="7.5" customHeight="1">
+    <row r="36" spans="1:7" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="37"/>
-      <c r="B36" s="200"/>
-      <c r="C36" s="201"/>
-      <c r="D36" s="202"/>
+      <c r="B36" s="99"/>
+      <c r="C36" s="100"/>
+      <c r="D36" s="101"/>
       <c r="E36" s="76"/>
       <c r="F36" s="39"/>
       <c r="G36" s="23"/>
     </row>
-    <row r="37" spans="1:7">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="37"/>
-      <c r="B37" s="179" t="s">
-        <v>85</v>
-      </c>
-      <c r="C37" s="180"/>
-      <c r="D37" s="181"/>
+      <c r="B37" s="118" t="s">
+        <v>79</v>
+      </c>
+      <c r="C37" s="119"/>
+      <c r="D37" s="120"/>
       <c r="E37" s="26"/>
       <c r="F37" s="2"/>
       <c r="G37" s="23"/>
     </row>
-    <row r="38" spans="1:7" ht="15.75" customHeight="1">
-      <c r="A38" s="163" t="s">
-        <v>101</v>
-      </c>
-      <c r="B38" s="164"/>
-      <c r="C38" s="165"/>
+    <row r="38" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="159" t="s">
+        <v>103</v>
+      </c>
+      <c r="B38" s="160"/>
+      <c r="C38" s="161"/>
       <c r="D38" s="58"/>
       <c r="E38" s="26"/>
       <c r="F38" s="2"/>
       <c r="G38" s="23"/>
     </row>
-    <row r="39" spans="1:7" ht="15.75">
-      <c r="A39" s="166"/>
-      <c r="B39" s="167"/>
-      <c r="C39" s="168"/>
-      <c r="D39" s="188" t="s">
-        <v>60</v>
-      </c>
-      <c r="E39" s="189"/>
+    <row r="39" spans="1:7" ht="15" x14ac:dyDescent="0.25">
+      <c r="A39" s="162"/>
+      <c r="B39" s="163"/>
+      <c r="C39" s="164"/>
+      <c r="D39" s="127" t="s">
+        <v>54</v>
+      </c>
+      <c r="E39" s="128"/>
       <c r="F39" s="30"/>
-      <c r="G39" s="9">
+      <c r="G39" s="9" t="e">
         <f>SUM(G28:G38)</f>
-        <v>437892.00000000006</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" ht="15.75">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A40" s="48" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="B40" s="44"/>
       <c r="C40" s="27"/>
-      <c r="D40" s="190" t="s">
-        <v>61</v>
-      </c>
-      <c r="E40" s="191"/>
+      <c r="D40" s="129" t="s">
+        <v>55</v>
+      </c>
+      <c r="E40" s="130"/>
       <c r="F40" s="30"/>
       <c r="G40" s="9">
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:7" ht="15.75" customHeight="1">
+    <row r="41" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="45" t="s">
+        <v>58</v>
+      </c>
+      <c r="B41" s="156" t="s">
         <v>64</v>
       </c>
-      <c r="B41" s="160" t="s">
-        <v>70</v>
-      </c>
-      <c r="C41" s="161"/>
-      <c r="D41" s="190" t="s">
-        <v>62</v>
-      </c>
-      <c r="E41" s="191"/>
+      <c r="C41" s="157"/>
+      <c r="D41" s="129" t="s">
+        <v>56</v>
+      </c>
+      <c r="E41" s="130"/>
       <c r="F41" s="30"/>
       <c r="G41" s="9">
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:7" ht="15.75" customHeight="1">
+    <row r="42" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="47" t="s">
+        <v>59</v>
+      </c>
+      <c r="B42" s="155" t="s">
+        <v>41</v>
+      </c>
+      <c r="C42" s="158"/>
+      <c r="D42" s="137" t="s">
+        <v>57</v>
+      </c>
+      <c r="E42" s="138"/>
+      <c r="F42" s="30"/>
+      <c r="G42" s="75" t="e">
+        <f>G39-G40-G41</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="47" t="s">
+        <v>60</v>
+      </c>
+      <c r="B43" s="155" t="s">
+        <v>40</v>
+      </c>
+      <c r="C43" s="155"/>
+      <c r="D43" s="131" t="s">
         <v>65</v>
       </c>
-      <c r="B42" s="159" t="s">
-        <v>41</v>
-      </c>
-      <c r="C42" s="162"/>
-      <c r="D42" s="198" t="s">
+      <c r="E43" s="132"/>
+      <c r="F43" s="132"/>
+      <c r="G43" s="133"/>
+    </row>
+    <row r="44" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="47" t="s">
+        <v>61</v>
+      </c>
+      <c r="B44" s="155" t="s">
+        <v>66</v>
+      </c>
+      <c r="C44" s="155"/>
+      <c r="D44" s="134"/>
+      <c r="E44" s="135"/>
+      <c r="F44" s="135"/>
+      <c r="G44" s="136"/>
+    </row>
+    <row r="45" spans="1:7" ht="15" x14ac:dyDescent="0.25">
+      <c r="A45" s="47" t="s">
+        <v>62</v>
+      </c>
+      <c r="B45" s="154" t="s">
+        <v>42</v>
+      </c>
+      <c r="C45" s="154"/>
+      <c r="D45" s="121"/>
+      <c r="E45" s="122"/>
+      <c r="F45" s="122"/>
+      <c r="G45" s="123"/>
+    </row>
+    <row r="46" spans="1:7" ht="15" x14ac:dyDescent="0.25">
+      <c r="A46" s="46" t="s">
         <v>63</v>
       </c>
-      <c r="E42" s="199"/>
-      <c r="F42" s="30"/>
-      <c r="G42" s="75">
-        <f>G39-G40-G41</f>
-        <v>437892.00000000006</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7" ht="15.75" customHeight="1">
-      <c r="A43" s="47" t="s">
-        <v>66</v>
-      </c>
-      <c r="B43" s="159" t="s">
-        <v>40</v>
-      </c>
-      <c r="C43" s="159"/>
-      <c r="D43" s="192" t="s">
-        <v>71</v>
-      </c>
-      <c r="E43" s="193"/>
-      <c r="F43" s="193"/>
-      <c r="G43" s="194"/>
-    </row>
-    <row r="44" spans="1:7" ht="15.75" customHeight="1">
-      <c r="A44" s="47" t="s">
-        <v>67</v>
-      </c>
-      <c r="B44" s="159" t="s">
+      <c r="B46" s="149" t="s">
+        <v>43</v>
+      </c>
+      <c r="C46" s="149"/>
+      <c r="D46" s="121"/>
+      <c r="E46" s="122"/>
+      <c r="F46" s="122"/>
+      <c r="G46" s="123"/>
+    </row>
+    <row r="47" spans="1:7" ht="15" x14ac:dyDescent="0.25">
+      <c r="A47" s="112" t="s">
+        <v>73</v>
+      </c>
+      <c r="B47" s="113"/>
+      <c r="C47" s="114"/>
+      <c r="D47" s="121"/>
+      <c r="E47" s="122"/>
+      <c r="F47" s="122"/>
+      <c r="G47" s="123"/>
+    </row>
+    <row r="48" spans="1:7" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="115" t="s">
         <v>72</v>
       </c>
-      <c r="C44" s="159"/>
-      <c r="D44" s="195"/>
-      <c r="E44" s="196"/>
-      <c r="F44" s="196"/>
-      <c r="G44" s="197"/>
-    </row>
-    <row r="45" spans="1:7" ht="15.75">
-      <c r="A45" s="47" t="s">
-        <v>68</v>
-      </c>
-      <c r="B45" s="158" t="s">
-        <v>42</v>
-      </c>
-      <c r="C45" s="158"/>
-      <c r="D45" s="182"/>
-      <c r="E45" s="183"/>
-      <c r="F45" s="183"/>
-      <c r="G45" s="184"/>
-    </row>
-    <row r="46" spans="1:7" ht="15.75">
-      <c r="A46" s="46" t="s">
-        <v>69</v>
-      </c>
-      <c r="B46" s="153" t="s">
-        <v>43</v>
-      </c>
-      <c r="C46" s="153"/>
-      <c r="D46" s="182"/>
-      <c r="E46" s="183"/>
-      <c r="F46" s="183"/>
-      <c r="G46" s="184"/>
-    </row>
-    <row r="47" spans="1:7" ht="15.75">
-      <c r="A47" s="173" t="s">
-        <v>79</v>
-      </c>
-      <c r="B47" s="174"/>
-      <c r="C47" s="175"/>
-      <c r="D47" s="182"/>
-      <c r="E47" s="183"/>
-      <c r="F47" s="183"/>
-      <c r="G47" s="184"/>
-    </row>
-    <row r="48" spans="1:7" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A48" s="176" t="s">
-        <v>78</v>
-      </c>
-      <c r="B48" s="177"/>
-      <c r="C48" s="178"/>
-      <c r="D48" s="185" t="s">
+      <c r="B48" s="116"/>
+      <c r="C48" s="117"/>
+      <c r="D48" s="124" t="s">
         <v>15</v>
       </c>
-      <c r="E48" s="186"/>
-      <c r="F48" s="186"/>
-      <c r="G48" s="187"/>
+      <c r="E48" s="125"/>
+      <c r="F48" s="125"/>
+      <c r="G48" s="126"/>
     </row>
   </sheetData>
   <mergeCells count="73">
-    <mergeCell ref="C21:G21"/>
-    <mergeCell ref="C22:G22"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A22:B23"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="C24:G24"/>
-    <mergeCell ref="B35:D35"/>
-    <mergeCell ref="B36:D36"/>
-    <mergeCell ref="A27:A29"/>
-    <mergeCell ref="B31:D31"/>
-    <mergeCell ref="B32:D32"/>
-    <mergeCell ref="B33:D33"/>
-    <mergeCell ref="B34:D34"/>
-    <mergeCell ref="A47:C47"/>
-    <mergeCell ref="A48:C48"/>
-    <mergeCell ref="B37:D37"/>
-    <mergeCell ref="D47:G47"/>
-    <mergeCell ref="D48:G48"/>
-    <mergeCell ref="D39:E39"/>
-    <mergeCell ref="D40:E40"/>
-    <mergeCell ref="D41:E41"/>
-    <mergeCell ref="D43:G44"/>
-    <mergeCell ref="D42:E42"/>
-    <mergeCell ref="D45:G45"/>
-    <mergeCell ref="D46:G46"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="E2:G2"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="E4:G4"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="C6:G6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="C7:G7"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="C8:G8"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="C9:G9"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="C10:G10"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="C11:G11"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="C12:G12"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="C13:G13"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="C14:G14"/>
+    <mergeCell ref="C17:G17"/>
+    <mergeCell ref="C18:G18"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="C15:G15"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="C16:G16"/>
     <mergeCell ref="C19:G19"/>
     <mergeCell ref="C20:G20"/>
     <mergeCell ref="C23:G23"/>
@@ -2915,37 +2953,32 @@
     <mergeCell ref="A38:C39"/>
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="C30:D30"/>
-    <mergeCell ref="C17:G17"/>
-    <mergeCell ref="C18:G18"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="C15:G15"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="C16:G16"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="C12:G12"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="C13:G13"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="C14:G14"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="C9:G9"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="C10:G10"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="C11:G11"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="C6:G6"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="C7:G7"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="C8:G8"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="E2:G2"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="E4:G4"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="E5:G5"/>
-    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A47:C47"/>
+    <mergeCell ref="A48:C48"/>
+    <mergeCell ref="B37:D37"/>
+    <mergeCell ref="D47:G47"/>
+    <mergeCell ref="D48:G48"/>
+    <mergeCell ref="D39:E39"/>
+    <mergeCell ref="D40:E40"/>
+    <mergeCell ref="D41:E41"/>
+    <mergeCell ref="D43:G44"/>
+    <mergeCell ref="D42:E42"/>
+    <mergeCell ref="D45:G45"/>
+    <mergeCell ref="D46:G46"/>
+    <mergeCell ref="B35:D35"/>
+    <mergeCell ref="B36:D36"/>
+    <mergeCell ref="A27:A29"/>
+    <mergeCell ref="B31:D31"/>
+    <mergeCell ref="B32:D32"/>
+    <mergeCell ref="B33:D33"/>
+    <mergeCell ref="B34:D34"/>
+    <mergeCell ref="C21:G21"/>
+    <mergeCell ref="C22:G22"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A22:B23"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="C24:G24"/>
   </mergeCells>
   <pageMargins left="3.9370078740157501E-2" right="3.9370078740157501E-2" top="1.69291338582677" bottom="0.31496062992126" header="7.8740157480315001E-2" footer="7.8740157480315001E-2"/>
   <pageSetup paperSize="9" scale="90" orientation="portrait" r:id="rId1"/>
@@ -2956,321 +2989,327 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:M44"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="23.125" customWidth="1"/>
-    <col min="3" max="3" width="9.375" customWidth="1"/>
-    <col min="4" max="4" width="13.875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.25" customWidth="1"/>
-    <col min="6" max="6" width="12.125" customWidth="1"/>
+    <col min="2" max="2" width="23.09765625" customWidth="1"/>
+    <col min="3" max="3" width="9.3984375" customWidth="1"/>
+    <col min="4" max="4" width="13.8984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.19921875" customWidth="1"/>
+    <col min="6" max="6" width="12.09765625" customWidth="1"/>
     <col min="7" max="7" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="35.25" thickBot="1">
-      <c r="A1" s="232" t="s">
+    <row r="1" spans="1:13" ht="35.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="280" t="s">
         <v>34</v>
       </c>
-      <c r="B1" s="232"/>
-      <c r="C1" s="232"/>
-      <c r="D1" s="232"/>
-      <c r="E1" s="232"/>
-      <c r="F1" s="232"/>
-      <c r="G1" s="232"/>
-    </row>
-    <row r="2" spans="1:13" ht="18.75" thickBot="1">
+      <c r="B1" s="280"/>
+      <c r="C1" s="280"/>
+      <c r="D1" s="280"/>
+      <c r="E1" s="280"/>
+      <c r="F1" s="280"/>
+      <c r="G1" s="280"/>
+    </row>
+    <row r="2" spans="1:13" ht="18" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="10" t="s">
         <v>14</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
-      <c r="E2" s="233" t="s">
-        <v>81</v>
-      </c>
-      <c r="F2" s="234"/>
-      <c r="G2" s="235"/>
-      <c r="K2" s="233" t="s">
-        <v>81</v>
-      </c>
-      <c r="L2" s="234"/>
-      <c r="M2" s="235"/>
-    </row>
-    <row r="3" spans="1:13" ht="15" thickBot="1">
-      <c r="A3" s="95" t="s">
-        <v>73</v>
-      </c>
-      <c r="B3" s="95"/>
-      <c r="C3" s="95"/>
-      <c r="D3" s="95"/>
-      <c r="E3" s="95"/>
-      <c r="F3" s="95"/>
-      <c r="G3" s="96"/>
-    </row>
-    <row r="4" spans="1:13" ht="16.5">
+      <c r="E2" s="231" t="s">
+        <v>75</v>
+      </c>
+      <c r="F2" s="232"/>
+      <c r="G2" s="233"/>
+      <c r="K2" s="231" t="s">
+        <v>75</v>
+      </c>
+      <c r="L2" s="232"/>
+      <c r="M2" s="233"/>
+    </row>
+    <row r="3" spans="1:13" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="226" t="s">
+        <v>67</v>
+      </c>
+      <c r="B3" s="226"/>
+      <c r="C3" s="226"/>
+      <c r="D3" s="226"/>
+      <c r="E3" s="226"/>
+      <c r="F3" s="226"/>
+      <c r="G3" s="227"/>
+    </row>
+    <row r="4" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B4" s="77" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="240" t="s">
-        <v>74</v>
-      </c>
-      <c r="D4" s="241"/>
-      <c r="E4" s="242"/>
-      <c r="F4" s="236" t="s">
+      <c r="C4" s="285" t="s">
+        <v>68</v>
+      </c>
+      <c r="D4" s="286"/>
+      <c r="E4" s="287"/>
+      <c r="F4" s="281" t="s">
         <v>3</v>
       </c>
-      <c r="G4" s="237"/>
-    </row>
-    <row r="5" spans="1:13" ht="16.5">
+      <c r="G4" s="282"/>
+    </row>
+    <row r="5" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>4</v>
       </c>
       <c r="B5" s="79" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="243" t="s">
-        <v>95</v>
-      </c>
-      <c r="D5" s="244"/>
-      <c r="E5" s="245"/>
-      <c r="F5" s="238" t="s">
-        <v>96</v>
-      </c>
-      <c r="G5" s="239"/>
-    </row>
-    <row r="6" spans="1:13" ht="15.75">
-      <c r="A6" s="97" t="s">
+      <c r="C5" s="288" t="s">
+        <v>98</v>
+      </c>
+      <c r="D5" s="289"/>
+      <c r="E5" s="290"/>
+      <c r="F5" s="283" t="s">
+        <v>114</v>
+      </c>
+      <c r="G5" s="284"/>
+    </row>
+    <row r="6" spans="1:13" ht="15" x14ac:dyDescent="0.25">
+      <c r="A6" s="182" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="98"/>
-      <c r="C6" s="99" t="s">
+      <c r="B6" s="185"/>
+      <c r="C6" s="205" t="s">
         <v>19</v>
       </c>
-      <c r="D6" s="100"/>
-      <c r="E6" s="100"/>
-      <c r="F6" s="100"/>
-      <c r="G6" s="101"/>
-    </row>
-    <row r="7" spans="1:13" ht="15.75">
-      <c r="A7" s="102" t="s">
+      <c r="D6" s="206"/>
+      <c r="E6" s="206"/>
+      <c r="F6" s="206"/>
+      <c r="G6" s="207"/>
+    </row>
+    <row r="7" spans="1:13" ht="15" x14ac:dyDescent="0.25">
+      <c r="A7" s="208" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="103"/>
-      <c r="C7" s="104" t="s">
-        <v>55</v>
-      </c>
-      <c r="D7" s="105"/>
-      <c r="E7" s="105"/>
-      <c r="F7" s="105"/>
-      <c r="G7" s="106"/>
+      <c r="B7" s="209"/>
+      <c r="C7" s="210" t="s">
+        <v>108</v>
+      </c>
+      <c r="D7" s="211"/>
+      <c r="E7" s="211"/>
+      <c r="F7" s="211"/>
+      <c r="G7" s="212"/>
       <c r="H7" s="25"/>
       <c r="I7" s="24"/>
     </row>
-    <row r="8" spans="1:13">
-      <c r="A8" s="107" t="s">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A8" s="195" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="108"/>
-      <c r="C8" s="109"/>
-      <c r="D8" s="110"/>
-      <c r="E8" s="110"/>
-      <c r="F8" s="110"/>
-      <c r="G8" s="111"/>
-    </row>
-    <row r="9" spans="1:13" ht="15.75">
-      <c r="A9" s="107" t="s">
+      <c r="B8" s="110"/>
+      <c r="C8" s="202"/>
+      <c r="D8" s="203"/>
+      <c r="E8" s="203"/>
+      <c r="F8" s="203"/>
+      <c r="G8" s="204"/>
+    </row>
+    <row r="9" spans="1:13" ht="15" x14ac:dyDescent="0.25">
+      <c r="A9" s="195" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="112"/>
-      <c r="C9" s="113" t="s">
+      <c r="B9" s="111"/>
+      <c r="C9" s="196" t="s">
         <v>22</v>
       </c>
-      <c r="D9" s="114"/>
-      <c r="E9" s="114"/>
-      <c r="F9" s="114"/>
-      <c r="G9" s="115"/>
-    </row>
-    <row r="10" spans="1:13" ht="15.75">
-      <c r="A10" s="107" t="s">
+      <c r="D9" s="197"/>
+      <c r="E9" s="197"/>
+      <c r="F9" s="197"/>
+      <c r="G9" s="198"/>
+    </row>
+    <row r="10" spans="1:13" ht="15" x14ac:dyDescent="0.25">
+      <c r="A10" s="195" t="s">
         <v>21</v>
       </c>
-      <c r="B10" s="112"/>
-      <c r="C10" s="116" t="s">
-        <v>107</v>
-      </c>
-      <c r="D10" s="117"/>
-      <c r="E10" s="117"/>
-      <c r="F10" s="117"/>
-      <c r="G10" s="118"/>
-    </row>
-    <row r="11" spans="1:13">
-      <c r="A11" s="107" t="s">
+      <c r="B10" s="111"/>
+      <c r="C10" s="199" t="s">
+        <v>96</v>
+      </c>
+      <c r="D10" s="200"/>
+      <c r="E10" s="200"/>
+      <c r="F10" s="200"/>
+      <c r="G10" s="201"/>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A11" s="195" t="s">
         <v>23</v>
       </c>
-      <c r="B11" s="112"/>
-      <c r="C11" s="109"/>
-      <c r="D11" s="110"/>
-      <c r="E11" s="110"/>
-      <c r="F11" s="110"/>
-      <c r="G11" s="111"/>
-    </row>
-    <row r="12" spans="1:13">
-      <c r="A12" s="97" t="s">
+      <c r="B11" s="111"/>
+      <c r="C11" s="202"/>
+      <c r="D11" s="203"/>
+      <c r="E11" s="203"/>
+      <c r="F11" s="203"/>
+      <c r="G11" s="204"/>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A12" s="182" t="s">
         <v>24</v>
       </c>
-      <c r="B12" s="119"/>
-      <c r="C12" s="120" t="s">
+      <c r="B12" s="183"/>
+      <c r="C12" s="184" t="s">
         <v>25</v>
       </c>
-      <c r="D12" s="98"/>
-      <c r="E12" s="98"/>
-      <c r="F12" s="98"/>
-      <c r="G12" s="121"/>
-    </row>
-    <row r="13" spans="1:13" ht="16.5" customHeight="1">
-      <c r="A13" s="122" t="s">
-        <v>49</v>
-      </c>
-      <c r="B13" s="123"/>
-      <c r="C13" s="124" t="s">
-        <v>44</v>
-      </c>
-      <c r="D13" s="125"/>
-      <c r="E13" s="125"/>
-      <c r="F13" s="125"/>
-      <c r="G13" s="126"/>
-    </row>
-    <row r="14" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A14" s="127" t="s">
-        <v>45</v>
-      </c>
-      <c r="B14" s="128"/>
-      <c r="C14" s="129" t="s">
-        <v>46</v>
-      </c>
-      <c r="D14" s="130"/>
-      <c r="E14" s="130"/>
-      <c r="F14" s="130"/>
-      <c r="G14" s="131"/>
-    </row>
-    <row r="15" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A15" s="138" t="s">
+      <c r="D12" s="185"/>
+      <c r="E12" s="185"/>
+      <c r="F12" s="185"/>
+      <c r="G12" s="186"/>
+    </row>
+    <row r="13" spans="1:13" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="187" t="str">
+        <f>'Tax Invoice'!A13:B13</f>
+        <v>{{CONSIGNEE}}</v>
+      </c>
+      <c r="B13" s="188"/>
+      <c r="C13" s="189" t="str">
+        <f>'Tax Invoice'!C13:G13</f>
+        <v>{{NOTIFY_APPLICANT}}</v>
+      </c>
+      <c r="D13" s="190"/>
+      <c r="E13" s="190"/>
+      <c r="F13" s="190"/>
+      <c r="G13" s="191"/>
+    </row>
+    <row r="14" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="180" t="str">
+        <f>'Tax Invoice'!A14:B14</f>
+        <v>{{CONSIGNEE_ADDRESS}}</v>
+      </c>
+      <c r="B14" s="181"/>
+      <c r="C14" s="192" t="str">
+        <f>'Tax Invoice'!C14:G14</f>
+        <v>{{NOTIFY_APPLICANT_ADDRESS}}</v>
+      </c>
+      <c r="D14" s="193"/>
+      <c r="E14" s="193"/>
+      <c r="F14" s="193"/>
+      <c r="G14" s="194"/>
+    </row>
+    <row r="15" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="175" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="139"/>
-      <c r="C15" s="140" t="s">
-        <v>47</v>
-      </c>
-      <c r="D15" s="141"/>
-      <c r="E15" s="141"/>
-      <c r="F15" s="141"/>
-      <c r="G15" s="142"/>
-    </row>
-    <row r="16" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A16" s="127"/>
-      <c r="B16" s="128"/>
-      <c r="C16" s="140" t="s">
-        <v>48</v>
-      </c>
-      <c r="D16" s="141"/>
-      <c r="E16" s="141"/>
-      <c r="F16" s="141"/>
-      <c r="G16" s="142"/>
-    </row>
-    <row r="17" spans="1:7">
+      <c r="B15" s="176"/>
+      <c r="C15" s="177" t="str">
+        <f>'Tax Invoice'!C15:G15</f>
+        <v>PAN NO: {{PAN_NO}}</v>
+      </c>
+      <c r="D15" s="178"/>
+      <c r="E15" s="178"/>
+      <c r="F15" s="178"/>
+      <c r="G15" s="179"/>
+    </row>
+    <row r="16" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="180"/>
+      <c r="B16" s="181"/>
+      <c r="C16" s="177" t="str">
+        <f>'Tax Invoice'!C16:G16</f>
+        <v>EXIM CODE : {{EXIM_CODE}}</v>
+      </c>
+      <c r="D16" s="178"/>
+      <c r="E16" s="178"/>
+      <c r="F16" s="178"/>
+      <c r="G16" s="179"/>
+    </row>
+    <row r="17" spans="1:7" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A17" s="71" t="s">
         <v>26</v>
       </c>
       <c r="B17" s="49" t="s">
         <v>27</v>
       </c>
-      <c r="C17" s="132" t="s">
+      <c r="C17" s="169" t="s">
         <v>31</v>
       </c>
-      <c r="D17" s="133"/>
-      <c r="E17" s="133"/>
-      <c r="F17" s="133"/>
-      <c r="G17" s="134"/>
-    </row>
-    <row r="18" spans="1:7" ht="42.75" customHeight="1">
+      <c r="D17" s="170"/>
+      <c r="E17" s="170"/>
+      <c r="F17" s="170"/>
+      <c r="G17" s="171"/>
+    </row>
+    <row r="18" spans="1:7" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="41" t="s">
         <v>30</v>
       </c>
       <c r="B18" s="50" t="s">
-        <v>56</v>
-      </c>
-      <c r="C18" s="135" t="s">
-        <v>90</v>
-      </c>
-      <c r="D18" s="136"/>
-      <c r="E18" s="136"/>
-      <c r="F18" s="136"/>
-      <c r="G18" s="137"/>
-    </row>
-    <row r="19" spans="1:7">
+        <v>50</v>
+      </c>
+      <c r="C18" s="172" t="s">
+        <v>84</v>
+      </c>
+      <c r="D18" s="173"/>
+      <c r="E18" s="173"/>
+      <c r="F18" s="173"/>
+      <c r="G18" s="174"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="72" t="s">
         <v>28</v>
       </c>
       <c r="B19" s="73" t="s">
         <v>29</v>
       </c>
-      <c r="C19" s="266" t="s">
+      <c r="C19" s="274" t="s">
         <v>32</v>
       </c>
-      <c r="D19" s="267"/>
-      <c r="E19" s="267"/>
-      <c r="F19" s="267"/>
-      <c r="G19" s="268"/>
-    </row>
-    <row r="20" spans="1:7" ht="14.25" customHeight="1">
+      <c r="D19" s="275"/>
+      <c r="E19" s="275"/>
+      <c r="F19" s="275"/>
+      <c r="G19" s="276"/>
+    </row>
+    <row r="20" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="41" t="s">
         <v>6</v>
       </c>
       <c r="B20" s="78" t="s">
-        <v>45</v>
-      </c>
-      <c r="C20" s="269" t="s">
-        <v>54</v>
-      </c>
-      <c r="D20" s="270"/>
-      <c r="E20" s="270"/>
-      <c r="F20" s="270"/>
-      <c r="G20" s="271"/>
-    </row>
-    <row r="21" spans="1:7" ht="18.75" customHeight="1">
-      <c r="A21" s="279" t="s">
+        <v>44</v>
+      </c>
+      <c r="C20" s="247" t="s">
+        <v>49</v>
+      </c>
+      <c r="D20" s="248"/>
+      <c r="E20" s="248"/>
+      <c r="F20" s="248"/>
+      <c r="G20" s="249"/>
+    </row>
+    <row r="21" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="235" t="s">
         <v>9</v>
       </c>
-      <c r="B21" s="280"/>
-      <c r="C21" s="280"/>
-      <c r="D21" s="283" t="s">
-        <v>77</v>
-      </c>
-      <c r="E21" s="272" t="s">
-        <v>75</v>
-      </c>
-      <c r="F21" s="285" t="s">
-        <v>76</v>
-      </c>
-      <c r="G21" s="274" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" ht="20.25" customHeight="1">
-      <c r="A22" s="281"/>
-      <c r="B22" s="282"/>
-      <c r="C22" s="282"/>
-      <c r="D22" s="284"/>
-      <c r="E22" s="273"/>
-      <c r="F22" s="286"/>
-      <c r="G22" s="275"/>
-    </row>
-    <row r="23" spans="1:7" ht="15.75">
+      <c r="B21" s="236"/>
+      <c r="C21" s="236"/>
+      <c r="D21" s="239" t="s">
+        <v>71</v>
+      </c>
+      <c r="E21" s="250" t="s">
+        <v>69</v>
+      </c>
+      <c r="F21" s="241" t="s">
+        <v>70</v>
+      </c>
+      <c r="G21" s="252" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="237"/>
+      <c r="B22" s="238"/>
+      <c r="C22" s="238"/>
+      <c r="D22" s="240"/>
+      <c r="E22" s="251"/>
+      <c r="F22" s="242"/>
+      <c r="G22" s="253"/>
+    </row>
+    <row r="23" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A23" s="56"/>
       <c r="B23" s="57"/>
       <c r="C23" s="57"/>
@@ -3279,258 +3318,303 @@
       <c r="F23" s="55"/>
       <c r="G23" s="67"/>
     </row>
-    <row r="24" spans="1:7" ht="16.5" customHeight="1">
-      <c r="A24" s="264" t="s">
-        <v>91</v>
-      </c>
-      <c r="B24" s="265"/>
-      <c r="C24" s="265"/>
+    <row r="24" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="272" t="s">
+        <v>85</v>
+      </c>
+      <c r="B24" s="273"/>
+      <c r="C24" s="273"/>
       <c r="D24" s="61"/>
       <c r="E24" s="61"/>
       <c r="F24" s="59"/>
       <c r="G24" s="68"/>
     </row>
-    <row r="25" spans="1:7" ht="15.75">
-      <c r="A25" s="264" t="s">
-        <v>87</v>
-      </c>
-      <c r="B25" s="265"/>
-      <c r="C25" s="265"/>
+    <row r="25" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A25" s="272" t="s">
+        <v>81</v>
+      </c>
+      <c r="B25" s="273"/>
+      <c r="C25" s="273"/>
       <c r="D25" s="66" t="s">
-        <v>103</v>
-      </c>
-      <c r="E25" s="66">
-        <v>20812</v>
+        <v>111</v>
+      </c>
+      <c r="E25" s="66" t="s">
+        <v>112</v>
       </c>
       <c r="F25" s="65" t="s">
-        <v>104</v>
-      </c>
-      <c r="G25" s="69">
-        <v>42.28</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" ht="16.5">
-      <c r="A26" s="287" t="s">
         <v>93</v>
       </c>
-      <c r="B26" s="288"/>
-      <c r="C26" s="288"/>
+      <c r="G25" s="69" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A26" s="243" t="s">
+        <v>86</v>
+      </c>
+      <c r="B26" s="244"/>
+      <c r="C26" s="244"/>
       <c r="D26" s="62"/>
       <c r="E26" s="62"/>
       <c r="F26" s="54" t="s">
         <v>14</v>
       </c>
       <c r="G26" s="81" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" ht="15.75">
-      <c r="A27" s="289" t="s">
-        <v>102</v>
-      </c>
-      <c r="B27" s="290"/>
-      <c r="C27" s="290"/>
+        <v>94</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="15" x14ac:dyDescent="0.25">
+      <c r="A27" s="245" t="s">
+        <v>92</v>
+      </c>
+      <c r="B27" s="246"/>
+      <c r="C27" s="246"/>
       <c r="D27" s="66"/>
       <c r="E27" s="66"/>
       <c r="F27" s="65"/>
       <c r="G27" s="69"/>
     </row>
-    <row r="28" spans="1:7" ht="15.75">
-      <c r="A28" s="228"/>
-      <c r="B28" s="209"/>
-      <c r="C28" s="209"/>
+    <row r="28" spans="1:7" ht="15" x14ac:dyDescent="0.25">
+      <c r="A28" s="234"/>
+      <c r="B28" s="107"/>
+      <c r="C28" s="107"/>
       <c r="D28" s="66" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="E28" s="66">
         <v>20811</v>
       </c>
       <c r="F28" s="65" t="s">
-        <v>104</v>
+        <v>93</v>
       </c>
       <c r="G28" s="69">
         <v>41.93</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="16.5">
-      <c r="A29" s="107"/>
-      <c r="B29" s="108"/>
-      <c r="C29" s="108"/>
+    <row r="29" spans="1:7" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A29" s="195"/>
+      <c r="B29" s="110"/>
+      <c r="C29" s="110"/>
       <c r="D29" s="62"/>
       <c r="E29" s="62"/>
       <c r="F29" s="54" t="s">
         <v>14</v>
       </c>
       <c r="G29" s="81" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" ht="16.5">
-      <c r="A30" s="228" t="s">
-        <v>50</v>
-      </c>
-      <c r="B30" s="209"/>
-      <c r="C30" s="210"/>
+        <v>94</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A30" s="234" t="s">
+        <v>45</v>
+      </c>
+      <c r="B30" s="107"/>
+      <c r="C30" s="108"/>
       <c r="D30" s="53"/>
       <c r="E30" s="53"/>
       <c r="F30" s="59"/>
       <c r="G30" s="68"/>
     </row>
-    <row r="31" spans="1:7" ht="16.5" customHeight="1">
-      <c r="A31" s="228" t="s">
-        <v>58</v>
-      </c>
-      <c r="B31" s="209"/>
-      <c r="C31" s="210"/>
+    <row r="31" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="234" t="s">
+        <v>52</v>
+      </c>
+      <c r="B31" s="107"/>
+      <c r="C31" s="108"/>
       <c r="D31" s="66"/>
       <c r="E31" s="66"/>
       <c r="F31" s="65"/>
       <c r="G31" s="69"/>
     </row>
-    <row r="32" spans="1:7" ht="16.5">
-      <c r="A32" s="107" t="s">
-        <v>88</v>
-      </c>
-      <c r="B32" s="108"/>
-      <c r="C32" s="112"/>
+    <row r="32" spans="1:7" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A32" s="195" t="s">
+        <v>82</v>
+      </c>
+      <c r="B32" s="110"/>
+      <c r="C32" s="111"/>
       <c r="D32" s="62"/>
       <c r="E32" s="62"/>
       <c r="F32" s="54"/>
       <c r="G32" s="81"/>
     </row>
-    <row r="33" spans="1:7" ht="15.75">
-      <c r="A33" s="228" t="s">
-        <v>57</v>
-      </c>
-      <c r="B33" s="209"/>
-      <c r="C33" s="210"/>
+    <row r="33" spans="1:7" ht="15" x14ac:dyDescent="0.25">
+      <c r="A33" s="234" t="s">
+        <v>51</v>
+      </c>
+      <c r="B33" s="107"/>
+      <c r="C33" s="108"/>
       <c r="D33" s="66"/>
       <c r="E33" s="66"/>
       <c r="F33" s="65"/>
       <c r="G33" s="69"/>
     </row>
-    <row r="34" spans="1:7" ht="16.5" customHeight="1">
-      <c r="A34" s="276" t="s">
-        <v>83</v>
-      </c>
-      <c r="B34" s="277"/>
-      <c r="C34" s="278"/>
+    <row r="34" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="228" t="s">
+        <v>77</v>
+      </c>
+      <c r="B34" s="229"/>
+      <c r="C34" s="230"/>
       <c r="D34" s="63"/>
       <c r="E34" s="63"/>
       <c r="F34" s="54"/>
       <c r="G34" s="70"/>
     </row>
-    <row r="35" spans="1:7" ht="15.75">
-      <c r="A35" s="276" t="s">
-        <v>84</v>
-      </c>
-      <c r="B35" s="277"/>
-      <c r="C35" s="278"/>
+    <row r="35" spans="1:7" ht="15" x14ac:dyDescent="0.25">
+      <c r="A35" s="228" t="s">
+        <v>78</v>
+      </c>
+      <c r="B35" s="229"/>
+      <c r="C35" s="230"/>
       <c r="D35" s="66"/>
       <c r="E35" s="66"/>
       <c r="F35" s="65"/>
       <c r="G35" s="69"/>
     </row>
-    <row r="36" spans="1:7" ht="16.5">
-      <c r="A36" s="229"/>
-      <c r="B36" s="230"/>
-      <c r="C36" s="231"/>
+    <row r="36" spans="1:7" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A36" s="277"/>
+      <c r="B36" s="278"/>
+      <c r="C36" s="279"/>
       <c r="D36" s="64"/>
       <c r="E36" s="64"/>
       <c r="F36" s="54"/>
       <c r="G36" s="70"/>
     </row>
-    <row r="37" spans="1:7" ht="16.5">
-      <c r="A37" s="229"/>
-      <c r="B37" s="230"/>
-      <c r="C37" s="231"/>
+    <row r="37" spans="1:7" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A37" s="277"/>
+      <c r="B37" s="278"/>
+      <c r="C37" s="279"/>
       <c r="D37" s="66"/>
       <c r="E37" s="66"/>
       <c r="F37" s="65"/>
       <c r="G37" s="69"/>
     </row>
-    <row r="38" spans="1:7" ht="16.5">
-      <c r="A38" s="229"/>
-      <c r="B38" s="230"/>
-      <c r="C38" s="231"/>
+    <row r="38" spans="1:7" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A38" s="277"/>
+      <c r="B38" s="278"/>
+      <c r="C38" s="279"/>
       <c r="D38" s="64"/>
       <c r="E38" s="64"/>
       <c r="F38" s="54"/>
       <c r="G38" s="70"/>
     </row>
-    <row r="39" spans="1:7" ht="16.5">
-      <c r="A39" s="249"/>
-      <c r="B39" s="250"/>
-      <c r="C39" s="251"/>
-      <c r="D39" s="252" t="s">
-        <v>82</v>
-      </c>
-      <c r="E39" s="253"/>
-      <c r="F39" s="254"/>
+    <row r="39" spans="1:7" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A39" s="257"/>
+      <c r="B39" s="258"/>
+      <c r="C39" s="259"/>
+      <c r="D39" s="260" t="s">
+        <v>76</v>
+      </c>
+      <c r="E39" s="261"/>
+      <c r="F39" s="262"/>
       <c r="G39" s="74">
         <f>SUM(G23:G38)</f>
-        <v>84.210000000000008</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" ht="16.5">
+        <v>41.93</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" ht="16.8" x14ac:dyDescent="0.25">
       <c r="A40" s="11" t="s">
         <v>35</v>
       </c>
       <c r="B40" s="12"/>
       <c r="C40" s="12"/>
       <c r="D40" s="13"/>
-      <c r="E40" s="255" t="s">
-        <v>71</v>
-      </c>
-      <c r="F40" s="256"/>
-      <c r="G40" s="257"/>
-    </row>
-    <row r="41" spans="1:7" ht="16.5">
+      <c r="E40" s="263" t="s">
+        <v>65</v>
+      </c>
+      <c r="F40" s="264"/>
+      <c r="G40" s="265"/>
+    </row>
+    <row r="41" spans="1:7" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A41" s="14" t="s">
         <v>36</v>
       </c>
       <c r="B41" s="15"/>
       <c r="C41" s="15"/>
       <c r="D41" s="16"/>
-      <c r="E41" s="258"/>
-      <c r="F41" s="259"/>
-      <c r="G41" s="260"/>
-    </row>
-    <row r="42" spans="1:7" ht="16.5">
+      <c r="E41" s="266"/>
+      <c r="F41" s="267"/>
+      <c r="G41" s="268"/>
+    </row>
+    <row r="42" spans="1:7" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A42" s="14" t="s">
         <v>37</v>
       </c>
       <c r="B42" s="15"/>
       <c r="C42" s="15"/>
       <c r="D42" s="17"/>
-      <c r="E42" s="261"/>
-      <c r="F42" s="262"/>
-      <c r="G42" s="263"/>
-    </row>
-    <row r="43" spans="1:7" ht="16.5">
+      <c r="E42" s="269"/>
+      <c r="F42" s="270"/>
+      <c r="G42" s="271"/>
+    </row>
+    <row r="43" spans="1:7" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A43" s="14" t="s">
         <v>38</v>
       </c>
       <c r="B43" s="15"/>
       <c r="C43" s="15"/>
       <c r="D43" s="17"/>
-      <c r="E43" s="261"/>
-      <c r="F43" s="262"/>
-      <c r="G43" s="263"/>
-    </row>
-    <row r="44" spans="1:7" ht="17.25" thickBot="1">
+      <c r="E43" s="269"/>
+      <c r="F43" s="270"/>
+      <c r="G43" s="271"/>
+    </row>
+    <row r="44" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A44" s="18"/>
       <c r="B44" s="19"/>
       <c r="C44" s="20"/>
       <c r="D44" s="21"/>
-      <c r="E44" s="246" t="s">
+      <c r="E44" s="254" t="s">
         <v>39</v>
       </c>
-      <c r="F44" s="247"/>
-      <c r="G44" s="248"/>
+      <c r="F44" s="255"/>
+      <c r="G44" s="256"/>
     </row>
   </sheetData>
   <mergeCells count="61">
+    <mergeCell ref="A33:C33"/>
+    <mergeCell ref="A36:C36"/>
+    <mergeCell ref="A37:C37"/>
+    <mergeCell ref="A38:C38"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="E2:G2"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="C6:G6"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="C7:G7"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="C8:G8"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="C9:G9"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="C10:G10"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="C11:G11"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="C12:G12"/>
+    <mergeCell ref="E44:G44"/>
+    <mergeCell ref="A39:C39"/>
+    <mergeCell ref="D39:F39"/>
+    <mergeCell ref="E40:G40"/>
+    <mergeCell ref="E41:G41"/>
+    <mergeCell ref="E42:G42"/>
+    <mergeCell ref="E43:G43"/>
+    <mergeCell ref="C18:G18"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="A25:C25"/>
+    <mergeCell ref="C19:G19"/>
+    <mergeCell ref="C20:G20"/>
+    <mergeCell ref="E21:E22"/>
+    <mergeCell ref="G21:G22"/>
+    <mergeCell ref="C13:G13"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="C14:G14"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="C15:G15"/>
     <mergeCell ref="A34:C34"/>
     <mergeCell ref="A35:C35"/>
     <mergeCell ref="K2:M2"/>
@@ -3547,51 +3631,6 @@
     <mergeCell ref="A16:B16"/>
     <mergeCell ref="C16:G16"/>
     <mergeCell ref="C17:G17"/>
-    <mergeCell ref="C20:G20"/>
-    <mergeCell ref="E21:E22"/>
-    <mergeCell ref="G21:G22"/>
-    <mergeCell ref="C13:G13"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="C14:G14"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="C15:G15"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="C11:G11"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="C12:G12"/>
-    <mergeCell ref="E44:G44"/>
-    <mergeCell ref="A39:C39"/>
-    <mergeCell ref="D39:F39"/>
-    <mergeCell ref="E40:G40"/>
-    <mergeCell ref="E41:G41"/>
-    <mergeCell ref="E42:G42"/>
-    <mergeCell ref="E43:G43"/>
-    <mergeCell ref="C18:G18"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A24:C24"/>
-    <mergeCell ref="A25:C25"/>
-    <mergeCell ref="C19:G19"/>
-    <mergeCell ref="C8:G8"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="C9:G9"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="C10:G10"/>
-    <mergeCell ref="A33:C33"/>
-    <mergeCell ref="A36:C36"/>
-    <mergeCell ref="A37:C37"/>
-    <mergeCell ref="A38:C38"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="E2:G2"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="C6:G6"/>
-    <mergeCell ref="A3:G3"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="C7:G7"/>
-    <mergeCell ref="A8:B8"/>
   </mergeCells>
   <pageMargins left="0.1" right="0.1" top="1.69291338582677" bottom="0.31496062992126" header="0.196850393700787" footer="0.196850393700787"/>
   <pageSetup paperSize="9" scale="91" orientation="portrait" r:id="rId1"/>

</xml_diff>